<commit_message>
updated gumthalakadi gala galanu
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ITV PROGRAMMING\powerbi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2D2A3AFE-EAE6-47C4-A3B5-FAE72E2C9E4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C04E2D6C-D1EA-48F6-902F-8BB4BC992261}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{174AA38C-5DA2-4F67-8987-C75CBC84143F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
   <si>
     <t>productname</t>
   </si>
@@ -75,14 +75,25 @@
   </si>
   <si>
     <t>elect</t>
+  </si>
+  <si>
+    <t>qty</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -110,8 +121,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -446,21 +458,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{731DDD78-3800-4CD0-A96F-16139C9C2421}">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -468,10 +483,14 @@
         <v>10</v>
       </c>
       <c r="C2">
+        <f ca="1">RANDBETWEEN(3,10)</f>
+        <v>5</v>
+      </c>
+      <c r="D2">
         <v>7000</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -479,10 +498,14 @@
         <v>11</v>
       </c>
       <c r="C3">
+        <f t="shared" ref="C3:C8" ca="1" si="0">RANDBETWEEN(3,10)</f>
+        <v>3</v>
+      </c>
+      <c r="D3">
         <v>20000</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -490,10 +513,14 @@
         <v>10</v>
       </c>
       <c r="C4">
+        <f t="shared" ca="1" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="D4">
         <v>6200</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -501,10 +528,14 @@
         <v>11</v>
       </c>
       <c r="C5">
+        <f t="shared" ca="1" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="D5">
         <v>7800</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -512,10 +543,14 @@
         <v>10</v>
       </c>
       <c r="C6">
+        <f t="shared" ca="1" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="D6">
         <v>9000</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -523,10 +558,14 @@
         <v>10</v>
       </c>
       <c r="C7">
+        <f t="shared" ca="1" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="D7">
         <v>5615</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -534,6 +573,10 @@
         <v>10</v>
       </c>
       <c r="C8">
+        <f t="shared" ca="1" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="D8">
         <v>7090</v>
       </c>
     </row>

</xml_diff>